<commit_message>
n8n board refresh 2026-06-01T17:39:11Z
</commit_message>
<xml_diff>
--- a/app/reports/ACGP_research.xlsx
+++ b/app/reports/ACGP_research.xlsx
@@ -112,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -151,6 +151,8 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -618,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-05-30 22:16 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-01 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -862,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.0445300006866455</v>
+        <v>0.0447700023651123</v>
       </c>
     </row>
     <row r="6">
@@ -1417,7 +1419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1503,56 +1505,198 @@
         <v>14.99</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BETSF</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bit Brother Limited</t>
+        </is>
+      </c>
+      <c r="C6" s="32" t="n">
+        <v>124</v>
+      </c>
+      <c r="D6" s="33" t="n"/>
+      <c r="E6" s="33" t="n">
+        <v>0.129</v>
+      </c>
+      <c r="F6" s="33" t="n">
+        <v>-1.711</v>
+      </c>
+    </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Peer median</t>
-        </is>
-      </c>
-      <c r="D7" s="32">
-        <f>MEDIAN(D6:D5)</f>
-        <v/>
-      </c>
-      <c r="E7" s="32">
-        <f>MEDIAN(E6:E5)</f>
-        <v/>
-      </c>
-      <c r="F7" s="32">
-        <f>MEDIAN(F6:F5)</f>
-        <v/>
-      </c>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BGMO</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BERGAMO ACQUISITION CORP</t>
+        </is>
+      </c>
+      <c r="C7" s="32" t="n"/>
+      <c r="D7" s="33" t="n">
+        <v>4.0816326e-06</v>
+      </c>
+      <c r="E7" s="33" t="n"/>
+      <c r="F7" s="33" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Peer mean</t>
-        </is>
-      </c>
-      <c r="D8" s="32">
-        <f>AVERAGE(D6:D5)</f>
-        <v/>
-      </c>
-      <c r="E8" s="32">
-        <f>AVERAGE(E6:E5)</f>
-        <v/>
-      </c>
-      <c r="F8" s="32">
-        <f>AVERAGE(F6:F5)</f>
-        <v/>
-      </c>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>COWN</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>COWN</t>
+        </is>
+      </c>
+      <c r="C8" s="32" t="n"/>
+      <c r="D8" s="33" t="n"/>
+      <c r="E8" s="33" t="n"/>
+      <c r="F8" s="33" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Target percentile vs peers</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GHL</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>GHL</t>
+        </is>
+      </c>
+      <c r="C9" s="32" t="n"/>
       <c r="D9" s="33" t="n"/>
       <c r="E9" s="33" t="n"/>
       <c r="F9" s="33" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GRDI</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>GRDI</t>
+        </is>
+      </c>
+      <c r="C10" s="32" t="n"/>
+      <c r="D10" s="33" t="n"/>
+      <c r="E10" s="33" t="n"/>
+      <c r="F10" s="33" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LKADF</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>LKADF</t>
+        </is>
+      </c>
+      <c r="C11" s="32" t="n"/>
+      <c r="D11" s="33" t="n"/>
+      <c r="E11" s="33" t="n"/>
+      <c r="F11" s="33" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PROP</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Prairie Operating Co.</t>
+        </is>
+      </c>
+      <c r="C12" s="32" t="n">
+        <v>91623912</v>
+      </c>
+      <c r="D12" s="33" t="n"/>
+      <c r="E12" s="33" t="n">
+        <v>4.372</v>
+      </c>
+      <c r="F12" s="33" t="n">
+        <v>2.216</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RAFFF</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>RAFFF</t>
+        </is>
+      </c>
+      <c r="C13" s="32" t="n"/>
+      <c r="D13" s="33" t="n"/>
+      <c r="E13" s="33" t="n"/>
+      <c r="F13" s="33" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Peer median</t>
+        </is>
+      </c>
+      <c r="D15" s="34">
+        <f>MEDIAN(D6:D13)</f>
+        <v/>
+      </c>
+      <c r="E15" s="34">
+        <f>MEDIAN(E6:E13)</f>
+        <v/>
+      </c>
+      <c r="F15" s="34">
+        <f>MEDIAN(F6:F13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Peer mean</t>
+        </is>
+      </c>
+      <c r="D16" s="34">
+        <f>AVERAGE(D6:D13)</f>
+        <v/>
+      </c>
+      <c r="E16" s="34">
+        <f>AVERAGE(E6:E13)</f>
+        <v/>
+      </c>
+      <c r="F16" s="34">
+        <f>AVERAGE(F6:F13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Target percentile vs peers</t>
+        </is>
+      </c>
+      <c r="D17" s="35" t="n"/>
+      <c r="E17" s="35" t="n"/>
+      <c r="F17" s="35" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>(higher pct = more expensive than peers)</t>
         </is>

</xml_diff>

<commit_message>
n8n board refresh 2026-06-02T17:38:33Z
</commit_message>
<xml_diff>
--- a/app/reports/ACGP_research.xlsx
+++ b/app/reports/ACGP_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-01 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-02 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.929</v>
+        <v>0.93</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>37.25</v>
+        <v>37.21</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0.929</v>
+        <v>0.93</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.0447700023651123</v>
+        <v>0.04456999778747558</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>20648580.29530201</v>
+        <v>20648579.19914002</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>37.25</v>
+        <v>37.21</v>
       </c>
     </row>
     <row r="38">
@@ -1493,16 +1493,16 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>769159616</v>
+        <v>768333632</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>17.82</v>
+        <v>17.8</v>
       </c>
       <c r="E5" s="31" t="n">
-        <v>-27.59</v>
+        <v>-27.52</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>14.99</v>
+        <v>14.95</v>
       </c>
     </row>
     <row r="6">
@@ -1621,14 +1621,14 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>91623912</v>
+        <v>93822888</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n">
-        <v>4.372</v>
+        <v>4.4</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>2.216</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
n8n board refresh 2026-06-03T17:40:38Z
</commit_message>
<xml_diff>
--- a/app/reports/ACGP_research.xlsx
+++ b/app/reports/ACGP_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-02 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-03 17:37 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.93</v>
+        <v>0.931</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>37.21</v>
+        <v>37.15</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0.93</v>
+        <v>0.931</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04456999778747558</v>
+        <v>0.04497000217437744</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>20648579.19914002</v>
+        <v>20648580.99596231</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>37.21</v>
+        <v>37.15</v>
       </c>
     </row>
     <row r="38">
@@ -1493,16 +1493,16 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>768333632</v>
+        <v>767094784</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>17.8</v>
+        <v>17.78</v>
       </c>
       <c r="E5" s="31" t="n">
-        <v>-27.52</v>
+        <v>-27.47</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>14.95</v>
+        <v>14.92</v>
       </c>
     </row>
     <row r="6">
@@ -1621,14 +1621,14 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>93822888</v>
+        <v>94018352</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n">
-        <v>4.4</v>
+        <v>4.411</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>2.23</v>
+        <v>2.236</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
n8n board refresh 2026-06-04T17:39:30Z
</commit_message>
<xml_diff>
--- a/app/reports/ACGP_research.xlsx
+++ b/app/reports/ACGP_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-03 17:37 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-04 17:37 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04497000217437744</v>
+        <v>0.04470999717712403</v>
       </c>
     </row>
     <row r="6">
@@ -1499,10 +1499,10 @@
         <v>17.78</v>
       </c>
       <c r="E5" s="31" t="n">
-        <v>-27.47</v>
+        <v>-27.46</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>14.92</v>
+        <v>14.91</v>
       </c>
     </row>
     <row r="6">
@@ -1621,14 +1621,14 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>94018352</v>
+        <v>90920240</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n">
-        <v>4.411</v>
+        <v>4.381</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>2.236</v>
+        <v>2.221</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-28T17:39:55Z
</commit_message>
<xml_diff>
--- a/app/reports/ACGP_research.xlsx
+++ b/app/reports/ACGP_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-04 17:37 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-28 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.931</v>
+        <v>0.974</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>37.15</v>
+        <v>33.5</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0.931</v>
+        <v>0.974</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04470999717712403</v>
+        <v>0.04595999717712403</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>20648580.99596231</v>
+        <v>20648579.82089552</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>37.15</v>
+        <v>33.5</v>
       </c>
     </row>
     <row r="38">
@@ -1493,16 +1493,16 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>767094784</v>
+        <v>691727424</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>17.78</v>
+        <v>16.03</v>
       </c>
       <c r="E5" s="31" t="n">
-        <v>-27.46</v>
+        <v>-20.25</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>14.91</v>
+        <v>12.15</v>
       </c>
     </row>
     <row r="6">
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>124</v>
+        <v>62</v>
       </c>
       <c r="D6" s="33" t="n"/>
       <c r="E6" s="33" t="n">
@@ -1621,14 +1621,14 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>90920240</v>
+        <v>67992272</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n">
-        <v>4.381</v>
+        <v>4.274</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>2.221</v>
+        <v>2.167</v>
       </c>
     </row>
     <row r="13">

</xml_diff>